<commit_message>
Update GAE/NPC reports, Utilization, and 5-Year Trend
- Reports: Primary Comparison options per GAE menu, single-measure Monthly
  and Quarterly views with line charts and a Total column, per-type trend
  charts, Calendar Year pinned for last-year/monthly/quarterly views.
- Trend: GAE-only budget (SAP plan) and actuals, 2022-2025 actuals and
  2023-2025 budgets from the GAE past-years workbook.
- NPC report: sheet-style layout with committed amounts from S_ALR.
- Utilization: NPC IO figures from S_ALR, Group column from the NPC
  monitoring workbook, layout and spacing fixes.
- Migrations: npc_monitoring_io.group_name.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Budgeting System_Expense Line Items.xlsx
+++ b/Budgeting System_Expense Line Items.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jumalonpvp\Downloads\Budgeting System\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65C68696-F02D-4167-A840-5053809DCC5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8C8EB5D-6DAA-42BB-918F-8C4F4D8C7AA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7D30BD04-AED0-48C4-A0F0-DC51EF4C24C2}"/>
   </bookViews>
@@ -1420,9 +1420,6 @@
     <t>Princess Vera P. Jumalon</t>
   </si>
   <si>
-    <t>Daisy Abendanio</t>
-  </si>
-  <si>
     <t>Ma. Karen I. Caparas</t>
   </si>
   <si>
@@ -1562,6 +1559,9 @@
   </si>
   <si>
     <t>MTS Recovery</t>
+  </si>
+  <si>
+    <t>Daisy Abendanio, Albertine Ellen R. Jimenez</t>
   </si>
 </sst>
 </file>
@@ -2296,10 +2296,10 @@
         <v>453</v>
       </c>
       <c r="J3" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K3" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L3">
         <v>81123102</v>
@@ -2348,10 +2348,10 @@
         <v>453</v>
       </c>
       <c r="J4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L4">
         <v>81123102</v>
@@ -2400,10 +2400,10 @@
         <v>453</v>
       </c>
       <c r="J5" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K5" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L5">
         <v>81123102</v>
@@ -2454,10 +2454,10 @@
         <v>453</v>
       </c>
       <c r="J6" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="K6" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="L6">
         <v>81123102</v>
@@ -2502,10 +2502,10 @@
         <v>453</v>
       </c>
       <c r="J7" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="K7" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="L7">
         <v>80123102</v>
@@ -2546,10 +2546,10 @@
         <v>453</v>
       </c>
       <c r="J8" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="K8" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="L8">
         <v>80123102</v>
@@ -2584,10 +2584,10 @@
         <v>453</v>
       </c>
       <c r="J9" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="K9" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="L9">
         <v>80123102</v>
@@ -2624,10 +2624,10 @@
         <v>453</v>
       </c>
       <c r="J10" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="K10" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="L10">
         <v>80123102</v>
@@ -2670,10 +2670,10 @@
         <v>453</v>
       </c>
       <c r="J11" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K11" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L11">
         <v>81123102</v>
@@ -2722,10 +2722,10 @@
         <v>453</v>
       </c>
       <c r="J12" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="K12" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L12">
         <v>80123102</v>
@@ -2765,10 +2765,10 @@
         <v>453</v>
       </c>
       <c r="J13" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="K13" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L13">
         <v>80123102</v>
@@ -2854,10 +2854,10 @@
         <v>453</v>
       </c>
       <c r="J15" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K15" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L15">
         <v>80123102</v>
@@ -2897,10 +2897,10 @@
         <v>453</v>
       </c>
       <c r="J16" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K16" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L16">
         <v>81123102</v>
@@ -2949,10 +2949,10 @@
         <v>453</v>
       </c>
       <c r="J17" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K17" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L17">
         <v>81123102</v>
@@ -3001,10 +3001,10 @@
         <v>453</v>
       </c>
       <c r="J18" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K18" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L18">
         <v>81123102</v>
@@ -3047,10 +3047,10 @@
         <v>453</v>
       </c>
       <c r="J19" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K19" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L19">
         <v>81123102</v>
@@ -3093,10 +3093,10 @@
         <v>453</v>
       </c>
       <c r="J20" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="K20" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L20">
         <v>80123102</v>
@@ -3145,10 +3145,10 @@
         <v>453</v>
       </c>
       <c r="J21" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K21" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L21">
         <v>81123102</v>
@@ -3188,10 +3188,10 @@
         <v>453</v>
       </c>
       <c r="J22" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K22" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L22">
         <v>81123102</v>
@@ -3226,10 +3226,10 @@
         <v>453</v>
       </c>
       <c r="J23" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K23" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L23">
         <v>80123102</v>
@@ -3266,10 +3266,10 @@
         <v>453</v>
       </c>
       <c r="J24" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="K24" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L24">
         <v>80123102</v>
@@ -3309,10 +3309,10 @@
         <v>453</v>
       </c>
       <c r="J25" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K25" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L25">
         <v>81123102</v>
@@ -3349,10 +3349,10 @@
         <v>453</v>
       </c>
       <c r="J26" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K26" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L26">
         <v>81123102</v>
@@ -3392,10 +3392,10 @@
         <v>453</v>
       </c>
       <c r="J27" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K27" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L27">
         <v>81123102</v>
@@ -3435,10 +3435,10 @@
         <v>453</v>
       </c>
       <c r="J28" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K28" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L28">
         <v>81123102</v>
@@ -3481,10 +3481,10 @@
         <v>453</v>
       </c>
       <c r="J29" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K29" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L29">
         <v>80123102</v>
@@ -3521,10 +3521,10 @@
         <v>453</v>
       </c>
       <c r="J30" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K30" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L30">
         <v>80123102</v>
@@ -3570,10 +3570,10 @@
         <v>453</v>
       </c>
       <c r="J31" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K31" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L31">
         <v>81123102</v>
@@ -3622,10 +3622,10 @@
         <v>453</v>
       </c>
       <c r="J32" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K32" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L32">
         <v>81123102</v>
@@ -3665,10 +3665,10 @@
         <v>453</v>
       </c>
       <c r="J33" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K33" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L33">
         <v>81123102</v>
@@ -3706,10 +3706,10 @@
         <v>453</v>
       </c>
       <c r="J34" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K34" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L34" s="9">
         <v>80123102</v>
@@ -3746,10 +3746,10 @@
         <v>453</v>
       </c>
       <c r="J35" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="K35" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L35">
         <v>80123102</v>
@@ -3790,7 +3790,7 @@
         <v>264</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="I36" t="s">
         <v>445</v>
@@ -3825,10 +3825,10 @@
         <v>BCA-27-35</v>
       </c>
       <c r="E37" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="I37" t="s">
         <v>445</v>
@@ -3863,10 +3863,10 @@
         <v>BCA-27-36</v>
       </c>
       <c r="E38" t="s">
+        <v>503</v>
+      </c>
+      <c r="F38" s="5" t="s">
         <v>504</v>
-      </c>
-      <c r="F38" s="5" t="s">
-        <v>505</v>
       </c>
       <c r="I38" t="s">
         <v>445</v>
@@ -3901,10 +3901,10 @@
         <v>BCA-27-37</v>
       </c>
       <c r="E39" t="s">
+        <v>503</v>
+      </c>
+      <c r="F39" s="5" t="s">
         <v>504</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>505</v>
       </c>
       <c r="I39" t="s">
         <v>445</v>
@@ -3939,10 +3939,10 @@
         <v>BCA-27-38</v>
       </c>
       <c r="E40" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="F40" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="G40" s="5" t="s">
         <v>220</v>
@@ -3980,10 +3980,10 @@
         <v>BCA-27-39</v>
       </c>
       <c r="E41" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="F41" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="G41" s="5" t="s">
         <v>219</v>
@@ -4021,10 +4021,10 @@
         <v>BCA-27-40</v>
       </c>
       <c r="E42" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="F42" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="G42" s="5" t="s">
         <v>221</v>
@@ -4105,7 +4105,7 @@
         <v>306</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="I44" t="s">
         <v>445</v>
@@ -4353,10 +4353,10 @@
         <v>351</v>
       </c>
       <c r="J50" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K50" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L50">
         <v>90134102</v>
@@ -4394,10 +4394,10 @@
         <v>351</v>
       </c>
       <c r="J51" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K51" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L51">
         <v>90134102</v>
@@ -4439,10 +4439,10 @@
         <v>351</v>
       </c>
       <c r="J52" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K52" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L52">
         <v>90111101</v>
@@ -4474,7 +4474,7 @@
         <v>264</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="G53" s="5" t="s">
         <v>219</v>
@@ -4483,10 +4483,10 @@
         <v>351</v>
       </c>
       <c r="J53" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K53" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L53">
         <v>81134102</v>
@@ -4515,7 +4515,7 @@
         <v>264</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="G54" s="5" t="s">
         <v>221</v>
@@ -4524,10 +4524,10 @@
         <v>351</v>
       </c>
       <c r="J54" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K54" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L54">
         <v>90134102</v>
@@ -4565,10 +4565,10 @@
         <v>351</v>
       </c>
       <c r="J55" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K55" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L55">
         <v>80134102</v>
@@ -4609,10 +4609,10 @@
         <v>351</v>
       </c>
       <c r="J56" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K56" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L56">
         <v>81134102</v>
@@ -4653,10 +4653,10 @@
         <v>351</v>
       </c>
       <c r="J57" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K57" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L57">
         <v>90134102</v>
@@ -4697,10 +4697,10 @@
         <v>351</v>
       </c>
       <c r="J58" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K58" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L58">
         <v>80134102</v>
@@ -4741,10 +4741,10 @@
         <v>351</v>
       </c>
       <c r="J59" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K59" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L59">
         <v>81134102</v>
@@ -4785,10 +4785,10 @@
         <v>351</v>
       </c>
       <c r="J60" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K60" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L60">
         <v>90134102</v>
@@ -4829,10 +4829,10 @@
         <v>351</v>
       </c>
       <c r="J61" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K61" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L61">
         <v>90134102</v>
@@ -4873,10 +4873,10 @@
         <v>351</v>
       </c>
       <c r="J62" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K62" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L62">
         <v>80134102</v>
@@ -4911,10 +4911,10 @@
         <v>351</v>
       </c>
       <c r="J63" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K63" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L63">
         <v>90111101</v>
@@ -4952,10 +4952,10 @@
         <v>351</v>
       </c>
       <c r="J64" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K64" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L64">
         <v>90111101</v>
@@ -4996,10 +4996,10 @@
         <v>351</v>
       </c>
       <c r="J65" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K65" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L65">
         <v>80111101</v>
@@ -5040,10 +5040,10 @@
         <v>351</v>
       </c>
       <c r="J66" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K66" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L66">
         <v>81111101</v>
@@ -5084,10 +5084,10 @@
         <v>351</v>
       </c>
       <c r="J67" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K67" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L67">
         <v>80111101</v>
@@ -5128,10 +5128,10 @@
         <v>351</v>
       </c>
       <c r="J68" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K68" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L68">
         <v>81111101</v>
@@ -5169,10 +5169,10 @@
         <v>351</v>
       </c>
       <c r="J69" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K69" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L69">
         <v>81111101</v>
@@ -5210,10 +5210,10 @@
         <v>351</v>
       </c>
       <c r="J70" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K70" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L70">
         <v>81111101</v>
@@ -5254,10 +5254,10 @@
         <v>351</v>
       </c>
       <c r="J71" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K71" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L71">
         <v>80111101</v>
@@ -5298,10 +5298,10 @@
         <v>351</v>
       </c>
       <c r="J72" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K72" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L72">
         <v>81111101</v>
@@ -5342,10 +5342,10 @@
         <v>351</v>
       </c>
       <c r="J73" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K73" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L73">
         <v>90111101</v>
@@ -5374,19 +5374,19 @@
         <v>CF-27-25</v>
       </c>
       <c r="E74" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="F74" s="5" t="s">
         <v>483</v>
-      </c>
-      <c r="F74" s="5" t="s">
-        <v>484</v>
       </c>
       <c r="I74" t="s">
         <v>351</v>
       </c>
       <c r="J74" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K74" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L74">
         <v>90134102</v>
@@ -5412,19 +5412,19 @@
         <v>CF-27-26</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="I75" t="s">
         <v>351</v>
       </c>
       <c r="J75" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K75" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L75">
         <v>90134102</v>
@@ -5463,10 +5463,10 @@
         <v>351</v>
       </c>
       <c r="J76" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K76" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L76">
         <v>81134102</v>
@@ -5504,10 +5504,10 @@
         <v>351</v>
       </c>
       <c r="J77" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K77" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L77">
         <v>80134102</v>
@@ -5545,10 +5545,10 @@
         <v>351</v>
       </c>
       <c r="J78" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K78" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L78">
         <v>80134102</v>
@@ -5586,10 +5586,10 @@
         <v>351</v>
       </c>
       <c r="J79" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K79" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L79">
         <v>80134102</v>
@@ -5621,16 +5621,16 @@
         <v>313</v>
       </c>
       <c r="F80" s="5" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="I80" t="s">
         <v>351</v>
       </c>
       <c r="J80" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K80" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L80">
         <v>80134102</v>
@@ -5666,10 +5666,10 @@
         <v>165</v>
       </c>
       <c r="J81" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="K81" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="L81">
         <v>81314101</v>
@@ -5709,10 +5709,10 @@
         <v>165</v>
       </c>
       <c r="J82" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="K82" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="L82">
         <v>81314101</v>
@@ -5752,10 +5752,10 @@
         <v>165</v>
       </c>
       <c r="J83" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="K83" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="L83">
         <v>81314101</v>
@@ -5795,10 +5795,10 @@
         <v>165</v>
       </c>
       <c r="J84" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="K84" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="L84">
         <v>81314101</v>
@@ -5838,10 +5838,10 @@
         <v>165</v>
       </c>
       <c r="J85" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="K85" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="L85">
         <v>81314101</v>
@@ -5881,10 +5881,10 @@
         <v>165</v>
       </c>
       <c r="J86" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="K86" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="L86">
         <v>81314101</v>
@@ -5924,10 +5924,10 @@
         <v>165</v>
       </c>
       <c r="J87" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="K87" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="L87">
         <v>81314101</v>
@@ -5967,10 +5967,10 @@
         <v>165</v>
       </c>
       <c r="J88" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="K88" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="L88">
         <v>81314101</v>
@@ -6010,10 +6010,10 @@
         <v>165</v>
       </c>
       <c r="J89" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="K89" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="L89">
         <v>81314101</v>
@@ -6053,10 +6053,10 @@
         <v>353</v>
       </c>
       <c r="J90" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K90" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="L90">
         <v>80125101</v>
@@ -6094,10 +6094,10 @@
         <v>353</v>
       </c>
       <c r="J91" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K91" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="L91">
         <v>81125101</v>
@@ -6135,10 +6135,10 @@
         <v>353</v>
       </c>
       <c r="J92" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K92" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="L92">
         <v>90125101</v>
@@ -6173,10 +6173,10 @@
         <v>353</v>
       </c>
       <c r="J93" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K93" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="L93">
         <v>80125101</v>
@@ -6217,10 +6217,10 @@
         <v>353</v>
       </c>
       <c r="J94" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K94" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="L94">
         <v>80125101</v>
@@ -6258,10 +6258,10 @@
         <v>353</v>
       </c>
       <c r="J95" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K95" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="L95">
         <v>81125101</v>
@@ -6299,10 +6299,10 @@
         <v>353</v>
       </c>
       <c r="J96" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K96" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="L96">
         <v>90125101</v>
@@ -6338,10 +6338,10 @@
         <v>84</v>
       </c>
       <c r="J97" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K97" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L97">
         <v>81122101</v>
@@ -6381,10 +6381,10 @@
         <v>84</v>
       </c>
       <c r="J98" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K98" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L98">
         <v>81122101</v>
@@ -6424,10 +6424,10 @@
         <v>84</v>
       </c>
       <c r="J99" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K99" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L99">
         <v>81122101</v>
@@ -6467,10 +6467,10 @@
         <v>84</v>
       </c>
       <c r="J100" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K100" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L100">
         <v>81122101</v>
@@ -6510,10 +6510,10 @@
         <v>84</v>
       </c>
       <c r="J101" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K101" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L101">
         <v>81122101</v>
@@ -6553,10 +6553,10 @@
         <v>84</v>
       </c>
       <c r="J102" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K102" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L102">
         <v>81122101</v>
@@ -6596,10 +6596,10 @@
         <v>84</v>
       </c>
       <c r="J103" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K103" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L103">
         <v>81122101</v>
@@ -6639,10 +6639,10 @@
         <v>84</v>
       </c>
       <c r="J104" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K104" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L104">
         <v>81122101</v>
@@ -6682,10 +6682,10 @@
         <v>84</v>
       </c>
       <c r="J105" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K105" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L105">
         <v>81122101</v>
@@ -6725,10 +6725,10 @@
         <v>84</v>
       </c>
       <c r="J106" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K106" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L106">
         <v>81122101</v>
@@ -6768,10 +6768,10 @@
         <v>84</v>
       </c>
       <c r="J107" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K107" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L107">
         <v>81122101</v>
@@ -6811,10 +6811,10 @@
         <v>84</v>
       </c>
       <c r="J108" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K108" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L108">
         <v>81122101</v>
@@ -6854,10 +6854,10 @@
         <v>84</v>
       </c>
       <c r="J109" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K109" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L109">
         <v>81122101</v>
@@ -6897,10 +6897,10 @@
         <v>84</v>
       </c>
       <c r="J110" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K110" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L110">
         <v>81122101</v>
@@ -6940,10 +6940,10 @@
         <v>84</v>
       </c>
       <c r="J111" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K111" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L111">
         <v>81122101</v>
@@ -6983,10 +6983,10 @@
         <v>84</v>
       </c>
       <c r="J112" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K112" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L112">
         <v>81122101</v>
@@ -7026,10 +7026,10 @@
         <v>84</v>
       </c>
       <c r="J113" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K113" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L113">
         <v>81122101</v>
@@ -7069,10 +7069,10 @@
         <v>84</v>
       </c>
       <c r="J114" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K114" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L114">
         <v>81122101</v>
@@ -7112,10 +7112,10 @@
         <v>84</v>
       </c>
       <c r="J115" t="s">
-        <v>458</v>
+        <v>505</v>
       </c>
       <c r="K115" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L115">
         <v>81122101</v>
@@ -7155,10 +7155,10 @@
         <v>84</v>
       </c>
       <c r="J116" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="K116" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L116">
         <v>90122101</v>
@@ -7198,10 +7198,10 @@
         <v>84</v>
       </c>
       <c r="J117" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="K117" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L117">
         <v>90122101</v>
@@ -7240,11 +7240,11 @@
       <c r="I118" t="s">
         <v>84</v>
       </c>
-      <c r="J118" s="4" t="s">
-        <v>458</v>
+      <c r="J118" t="s">
+        <v>505</v>
       </c>
       <c r="K118" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L118">
         <v>81122101</v>
@@ -7292,11 +7292,11 @@
       <c r="I119" t="s">
         <v>84</v>
       </c>
-      <c r="J119" s="4" t="s">
-        <v>458</v>
+      <c r="J119" t="s">
+        <v>505</v>
       </c>
       <c r="K119" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L119">
         <v>81122101</v>
@@ -7335,11 +7335,11 @@
       <c r="I120" t="s">
         <v>84</v>
       </c>
-      <c r="J120" s="4" t="s">
-        <v>458</v>
+      <c r="J120" t="s">
+        <v>505</v>
       </c>
       <c r="K120" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L120">
         <v>81122101</v>
@@ -7387,11 +7387,11 @@
       <c r="I121" t="s">
         <v>84</v>
       </c>
-      <c r="J121" s="4" t="s">
-        <v>458</v>
+      <c r="J121" t="s">
+        <v>505</v>
       </c>
       <c r="K121" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L121">
         <v>81122101</v>
@@ -7441,11 +7441,11 @@
       <c r="I122" t="s">
         <v>84</v>
       </c>
-      <c r="J122" s="4" t="s">
-        <v>458</v>
+      <c r="J122" t="s">
+        <v>505</v>
       </c>
       <c r="K122" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L122">
         <v>90122101</v>
@@ -7495,11 +7495,11 @@
       <c r="I123" t="s">
         <v>84</v>
       </c>
-      <c r="J123" s="4" t="s">
-        <v>458</v>
+      <c r="J123" t="s">
+        <v>505</v>
       </c>
       <c r="K123" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L123">
         <v>81122101</v>
@@ -7549,11 +7549,11 @@
       <c r="I124" t="s">
         <v>84</v>
       </c>
-      <c r="J124" s="4" t="s">
-        <v>458</v>
+      <c r="J124" t="s">
+        <v>505</v>
       </c>
       <c r="K124" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L124">
         <v>80122101</v>
@@ -7601,11 +7601,11 @@
       <c r="I125" t="s">
         <v>84</v>
       </c>
-      <c r="J125" s="4" t="s">
-        <v>458</v>
+      <c r="J125" t="s">
+        <v>505</v>
       </c>
       <c r="K125" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L125">
         <v>81122101</v>
@@ -7653,11 +7653,11 @@
       <c r="I126" t="s">
         <v>84</v>
       </c>
-      <c r="J126" s="4" t="s">
-        <v>458</v>
+      <c r="J126" t="s">
+        <v>505</v>
       </c>
       <c r="K126" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L126">
         <v>81122101</v>
@@ -7705,11 +7705,11 @@
       <c r="I127" t="s">
         <v>84</v>
       </c>
-      <c r="J127" s="4" t="s">
-        <v>458</v>
+      <c r="J127" t="s">
+        <v>505</v>
       </c>
       <c r="K127" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L127">
         <v>81122101</v>
@@ -7757,11 +7757,11 @@
       <c r="I128" t="s">
         <v>84</v>
       </c>
-      <c r="J128" s="4" t="s">
-        <v>458</v>
+      <c r="J128" t="s">
+        <v>505</v>
       </c>
       <c r="K128" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L128">
         <v>81122101</v>
@@ -7809,11 +7809,11 @@
       <c r="I129" t="s">
         <v>84</v>
       </c>
-      <c r="J129" s="4" t="s">
-        <v>458</v>
+      <c r="J129" t="s">
+        <v>505</v>
       </c>
       <c r="K129" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L129">
         <v>81122101</v>
@@ -7861,11 +7861,11 @@
       <c r="I130" t="s">
         <v>84</v>
       </c>
-      <c r="J130" s="4" t="s">
-        <v>458</v>
+      <c r="J130" t="s">
+        <v>505</v>
       </c>
       <c r="K130" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L130">
         <v>81122101</v>
@@ -7907,11 +7907,11 @@
       <c r="I131" t="s">
         <v>84</v>
       </c>
-      <c r="J131" s="4" t="s">
-        <v>458</v>
+      <c r="J131" t="s">
+        <v>505</v>
       </c>
       <c r="K131" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L131">
         <v>81122101</v>
@@ -7950,11 +7950,11 @@
       <c r="I132" t="s">
         <v>84</v>
       </c>
-      <c r="J132" s="4" t="s">
-        <v>458</v>
+      <c r="J132" t="s">
+        <v>505</v>
       </c>
       <c r="K132" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L132">
         <v>81122101</v>
@@ -7993,11 +7993,11 @@
       <c r="I133" t="s">
         <v>84</v>
       </c>
-      <c r="J133" s="4" t="s">
-        <v>458</v>
+      <c r="J133" t="s">
+        <v>505</v>
       </c>
       <c r="K133" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L133">
         <v>81122101</v>
@@ -8045,11 +8045,11 @@
       <c r="I134" t="s">
         <v>84</v>
       </c>
-      <c r="J134" s="4" t="s">
-        <v>458</v>
+      <c r="J134" t="s">
+        <v>505</v>
       </c>
       <c r="K134" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L134">
         <v>81122101</v>
@@ -8099,11 +8099,11 @@
       <c r="I135" t="s">
         <v>84</v>
       </c>
-      <c r="J135" s="4" t="s">
-        <v>458</v>
+      <c r="J135" t="s">
+        <v>505</v>
       </c>
       <c r="K135" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L135">
         <v>90111101</v>
@@ -8153,11 +8153,11 @@
       <c r="I136" t="s">
         <v>84</v>
       </c>
-      <c r="J136" s="4" t="s">
-        <v>458</v>
+      <c r="J136" t="s">
+        <v>505</v>
       </c>
       <c r="K136" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L136">
         <v>80111101</v>
@@ -8204,11 +8204,11 @@
       <c r="I137" t="s">
         <v>84</v>
       </c>
-      <c r="J137" s="4" t="s">
-        <v>458</v>
+      <c r="J137" t="s">
+        <v>505</v>
       </c>
       <c r="K137" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L137">
         <v>81111101</v>
@@ -8253,11 +8253,11 @@
       <c r="I138" t="s">
         <v>84</v>
       </c>
-      <c r="J138" s="4" t="s">
-        <v>458</v>
+      <c r="J138" t="s">
+        <v>505</v>
       </c>
       <c r="K138" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L138">
         <v>81122101</v>
@@ -8299,11 +8299,11 @@
       <c r="I139" t="s">
         <v>84</v>
       </c>
-      <c r="J139" s="4" t="s">
-        <v>458</v>
+      <c r="J139" t="s">
+        <v>505</v>
       </c>
       <c r="K139" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L139">
         <v>81122101</v>
@@ -8351,11 +8351,11 @@
       <c r="I140" t="s">
         <v>84</v>
       </c>
-      <c r="J140" s="4" t="s">
-        <v>458</v>
+      <c r="J140" t="s">
+        <v>505</v>
       </c>
       <c r="K140" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L140">
         <v>90122101</v>
@@ -8384,7 +8384,7 @@
         <v>325</v>
       </c>
       <c r="F141" s="4" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G141" s="4" t="s">
         <v>221</v>
@@ -8394,10 +8394,10 @@
         <v>84</v>
       </c>
       <c r="J141" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K141" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L141">
         <v>90122101</v>
@@ -8429,7 +8429,7 @@
         <v>325</v>
       </c>
       <c r="F142" s="4" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G142" s="4" t="s">
         <v>219</v>
@@ -8439,10 +8439,10 @@
         <v>84</v>
       </c>
       <c r="J142" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K142" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L142">
         <v>81122101</v>
@@ -8474,7 +8474,7 @@
         <v>325</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G143" s="4" t="s">
         <v>220</v>
@@ -8484,10 +8484,10 @@
         <v>84</v>
       </c>
       <c r="J143" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K143" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L143">
         <v>80122101</v>
@@ -8524,10 +8524,10 @@
         <v>84</v>
       </c>
       <c r="J144" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K144" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L144">
         <v>90111101</v>
@@ -8567,10 +8567,10 @@
         <v>84</v>
       </c>
       <c r="J145" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K145" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L145">
         <v>90122101</v>
@@ -8610,10 +8610,10 @@
         <v>84</v>
       </c>
       <c r="J146" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K146" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L146">
         <v>90122101</v>
@@ -8650,10 +8650,10 @@
         <v>84</v>
       </c>
       <c r="J147" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K147" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L147">
         <v>90122101</v>
@@ -8691,10 +8691,10 @@
         <v>84</v>
       </c>
       <c r="J148" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K148" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L148">
         <v>90122101</v>
@@ -8736,10 +8736,10 @@
         <v>84</v>
       </c>
       <c r="J149" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K149" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L149">
         <v>80111101</v>
@@ -8781,10 +8781,10 @@
         <v>84</v>
       </c>
       <c r="J150" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K150" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L150">
         <v>90111101</v>
@@ -8826,10 +8826,10 @@
         <v>84</v>
       </c>
       <c r="J151" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K151" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L151">
         <v>81111101</v>
@@ -8868,11 +8868,11 @@
       <c r="I152" t="s">
         <v>84</v>
       </c>
-      <c r="J152" s="4" t="s">
-        <v>458</v>
+      <c r="J152" t="s">
+        <v>505</v>
       </c>
       <c r="K152" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L152">
         <v>81122101</v>
@@ -8911,11 +8911,11 @@
       <c r="I153" t="s">
         <v>84</v>
       </c>
-      <c r="J153" s="4" t="s">
-        <v>458</v>
+      <c r="J153" t="s">
+        <v>505</v>
       </c>
       <c r="K153" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L153">
         <v>81122101</v>
@@ -8954,11 +8954,11 @@
       <c r="I154" t="s">
         <v>84</v>
       </c>
-      <c r="J154" s="4" t="s">
-        <v>458</v>
+      <c r="J154" t="s">
+        <v>505</v>
       </c>
       <c r="K154" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L154">
         <v>81122101</v>
@@ -8997,11 +8997,11 @@
       <c r="I155" t="s">
         <v>84</v>
       </c>
-      <c r="J155" s="4" t="s">
-        <v>458</v>
+      <c r="J155" t="s">
+        <v>505</v>
       </c>
       <c r="K155" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L155">
         <v>81122101</v>
@@ -9037,11 +9037,11 @@
       <c r="I156" t="s">
         <v>84</v>
       </c>
-      <c r="J156" s="4" t="s">
-        <v>458</v>
+      <c r="J156" t="s">
+        <v>505</v>
       </c>
       <c r="K156" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L156">
         <v>81122101</v>
@@ -9080,11 +9080,11 @@
       <c r="I157" t="s">
         <v>84</v>
       </c>
-      <c r="J157" s="4" t="s">
-        <v>458</v>
+      <c r="J157" t="s">
+        <v>505</v>
       </c>
       <c r="K157" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L157">
         <v>81122101</v>
@@ -9126,10 +9126,10 @@
         <v>84</v>
       </c>
       <c r="J158" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K158" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L158">
         <v>81122101</v>
@@ -9174,10 +9174,10 @@
         <v>84</v>
       </c>
       <c r="J159" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K159" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L159">
         <v>90122101</v>
@@ -9222,10 +9222,10 @@
         <v>84</v>
       </c>
       <c r="J160" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K160" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L160">
         <v>81111101</v>
@@ -9267,10 +9267,10 @@
         <v>84</v>
       </c>
       <c r="J161" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K161" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L161">
         <v>80111101</v>
@@ -9312,10 +9312,10 @@
         <v>84</v>
       </c>
       <c r="J162" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K162" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L162">
         <v>90111101</v>
@@ -9357,10 +9357,10 @@
         <v>84</v>
       </c>
       <c r="J163" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K163" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L163">
         <v>81111101</v>
@@ -9402,10 +9402,10 @@
         <v>84</v>
       </c>
       <c r="J164" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K164" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L164">
         <v>80111101</v>
@@ -9447,10 +9447,10 @@
         <v>84</v>
       </c>
       <c r="J165" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K165" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L165">
         <v>90111101</v>
@@ -9492,10 +9492,10 @@
         <v>84</v>
       </c>
       <c r="J166" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K166" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L166">
         <v>81111101</v>
@@ -9537,10 +9537,10 @@
         <v>84</v>
       </c>
       <c r="J167" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K167" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L167">
         <v>80111101</v>
@@ -9582,10 +9582,10 @@
         <v>84</v>
       </c>
       <c r="J168" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K168" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L168">
         <v>90111101</v>
@@ -9627,10 +9627,10 @@
         <v>84</v>
       </c>
       <c r="J169" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K169" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L169">
         <v>90111101</v>
@@ -9672,10 +9672,10 @@
         <v>84</v>
       </c>
       <c r="J170" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K170" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L170">
         <v>81111101</v>
@@ -9717,10 +9717,10 @@
         <v>84</v>
       </c>
       <c r="J171" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K171" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L171">
         <v>81111101</v>
@@ -9762,10 +9762,10 @@
         <v>84</v>
       </c>
       <c r="J172" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K172" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L172">
         <v>80111101</v>
@@ -9807,10 +9807,10 @@
         <v>84</v>
       </c>
       <c r="J173" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K173" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L173">
         <v>90111101</v>
@@ -9852,10 +9852,10 @@
         <v>84</v>
       </c>
       <c r="J174" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K174" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L174">
         <v>81111101</v>
@@ -9897,10 +9897,10 @@
         <v>84</v>
       </c>
       <c r="J175" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K175" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L175">
         <v>80111101</v>
@@ -9942,10 +9942,10 @@
         <v>84</v>
       </c>
       <c r="J176" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K176" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L176">
         <v>90111101</v>
@@ -9987,10 +9987,10 @@
         <v>84</v>
       </c>
       <c r="J177" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K177" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L177">
         <v>81111101</v>
@@ -10032,10 +10032,10 @@
         <v>84</v>
       </c>
       <c r="J178" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K178" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L178">
         <v>80111101</v>
@@ -10077,10 +10077,10 @@
         <v>84</v>
       </c>
       <c r="J179" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K179" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L179">
         <v>90111101</v>
@@ -10122,10 +10122,10 @@
         <v>84</v>
       </c>
       <c r="J180" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K180" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L180">
         <v>80111101</v>
@@ -10167,10 +10167,10 @@
         <v>84</v>
       </c>
       <c r="J181" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K181" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L181">
         <v>80111101</v>
@@ -10212,10 +10212,10 @@
         <v>84</v>
       </c>
       <c r="J182" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K182" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L182">
         <v>90111101</v>
@@ -10257,10 +10257,10 @@
         <v>84</v>
       </c>
       <c r="J183" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K183" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L183">
         <v>81111101</v>
@@ -10302,10 +10302,10 @@
         <v>84</v>
       </c>
       <c r="J184" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K184" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L184">
         <v>81111101</v>
@@ -10345,10 +10345,10 @@
         <v>84</v>
       </c>
       <c r="J185" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K185" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L185">
         <v>90111101</v>
@@ -10380,7 +10380,7 @@
         <v>265</v>
       </c>
       <c r="F186" s="4" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="G186" s="4"/>
       <c r="H186" s="4"/>
@@ -10388,10 +10388,10 @@
         <v>84</v>
       </c>
       <c r="J186" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K186" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L186">
         <v>90111101</v>
@@ -10429,10 +10429,10 @@
         <v>84</v>
       </c>
       <c r="J187" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K187" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L187">
         <v>80111101</v>
@@ -10473,10 +10473,10 @@
         <v>84</v>
       </c>
       <c r="J188" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K188" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L188">
         <v>90111101</v>
@@ -10518,10 +10518,10 @@
         <v>84</v>
       </c>
       <c r="J189" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K189" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L189">
         <v>90111101</v>
@@ -10563,10 +10563,10 @@
         <v>84</v>
       </c>
       <c r="J190" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K190" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L190">
         <v>90111101</v>
@@ -10608,10 +10608,10 @@
         <v>84</v>
       </c>
       <c r="J191" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K191" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L191">
         <v>81111101</v>
@@ -10653,10 +10653,10 @@
         <v>84</v>
       </c>
       <c r="J192" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K192" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L192">
         <v>80111101</v>
@@ -10698,10 +10698,10 @@
         <v>84</v>
       </c>
       <c r="J193" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K193" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L193">
         <v>90111101</v>
@@ -10739,10 +10739,10 @@
         <v>84</v>
       </c>
       <c r="J194" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K194" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L194">
         <v>81111101</v>
@@ -10780,10 +10780,10 @@
         <v>84</v>
       </c>
       <c r="J195" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K195" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L195">
         <v>80111101</v>
@@ -10821,10 +10821,10 @@
         <v>84</v>
       </c>
       <c r="J196" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K196" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L196">
         <v>90111101</v>
@@ -10866,10 +10866,10 @@
         <v>84</v>
       </c>
       <c r="J197" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K197" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L197">
         <v>81111101</v>
@@ -10911,10 +10911,10 @@
         <v>84</v>
       </c>
       <c r="J198" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K198" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L198">
         <v>80111101</v>
@@ -10956,10 +10956,10 @@
         <v>84</v>
       </c>
       <c r="J199" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K199" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L199">
         <v>90111101</v>
@@ -11001,10 +11001,10 @@
         <v>84</v>
       </c>
       <c r="J200" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K200" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L200">
         <v>81111101</v>
@@ -11046,10 +11046,10 @@
         <v>84</v>
       </c>
       <c r="J201" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K201" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L201">
         <v>80111101</v>
@@ -11091,10 +11091,10 @@
         <v>84</v>
       </c>
       <c r="J202" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K202" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L202">
         <v>90111101</v>
@@ -11136,10 +11136,10 @@
         <v>84</v>
       </c>
       <c r="J203" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K203" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L203">
         <v>81111101</v>
@@ -11181,10 +11181,10 @@
         <v>84</v>
       </c>
       <c r="J204" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K204" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L204">
         <v>80111101</v>
@@ -11226,10 +11226,10 @@
         <v>84</v>
       </c>
       <c r="J205" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K205" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L205">
         <v>90111101</v>
@@ -11267,10 +11267,10 @@
         <v>84</v>
       </c>
       <c r="J206" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K206" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L206">
         <v>81111101</v>
@@ -11308,10 +11308,10 @@
         <v>84</v>
       </c>
       <c r="J207" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K207" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L207">
         <v>80111101</v>
@@ -11349,10 +11349,10 @@
         <v>84</v>
       </c>
       <c r="J208" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K208" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L208">
         <v>90111101</v>
@@ -11390,10 +11390,10 @@
         <v>84</v>
       </c>
       <c r="J209" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K209" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L209">
         <v>81111101</v>
@@ -11434,10 +11434,10 @@
         <v>84</v>
       </c>
       <c r="J210" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K210" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L210">
         <v>80111101</v>
@@ -11478,10 +11478,10 @@
         <v>84</v>
       </c>
       <c r="J211" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K211" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L211">
         <v>90111101</v>
@@ -11522,10 +11522,10 @@
         <v>84</v>
       </c>
       <c r="J212" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K212" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L212">
         <v>80111101</v>
@@ -11566,10 +11566,10 @@
         <v>84</v>
       </c>
       <c r="J213" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="K213" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L213">
         <v>90111101</v>
@@ -11607,10 +11607,10 @@
         <v>84</v>
       </c>
       <c r="J214" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K214" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L214">
         <v>81122101</v>
@@ -11647,10 +11647,10 @@
         <v>84</v>
       </c>
       <c r="J215" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K215" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L215">
         <v>81122101</v>
@@ -11687,10 +11687,10 @@
         <v>84</v>
       </c>
       <c r="J216" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K216" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L216">
         <v>81122101</v>
@@ -11727,10 +11727,10 @@
         <v>84</v>
       </c>
       <c r="J217" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K217" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L217">
         <v>81122101</v>
@@ -11765,10 +11765,10 @@
         <v>84</v>
       </c>
       <c r="J218" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K218" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L218">
         <v>81122101</v>
@@ -11805,10 +11805,10 @@
         <v>84</v>
       </c>
       <c r="J219" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K219" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L219">
         <v>81122101</v>
@@ -11845,10 +11845,10 @@
         <v>84</v>
       </c>
       <c r="J220" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K220" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L220">
         <v>81122101</v>
@@ -11885,10 +11885,10 @@
         <v>84</v>
       </c>
       <c r="J221" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K221" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L221">
         <v>81122101</v>
@@ -11923,10 +11923,10 @@
         <v>84</v>
       </c>
       <c r="J222" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K222" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L222">
         <v>81134102</v>
@@ -11963,10 +11963,10 @@
         <v>84</v>
       </c>
       <c r="J223" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K223" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L223">
         <v>81122101</v>
@@ -11995,7 +11995,7 @@
         <v>267</v>
       </c>
       <c r="F224" s="4" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="G224" s="4"/>
       <c r="H224" s="4"/>
@@ -12003,10 +12003,10 @@
         <v>84</v>
       </c>
       <c r="J224" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K224" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L224">
         <v>81122101</v>
@@ -12043,10 +12043,10 @@
         <v>84</v>
       </c>
       <c r="J225" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="K225" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L225">
         <v>81122101</v>
@@ -12086,10 +12086,10 @@
         <v>84</v>
       </c>
       <c r="J226" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="K226" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L226">
         <v>81122101</v>
@@ -12129,10 +12129,10 @@
         <v>84</v>
       </c>
       <c r="J227" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="K227" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L227">
         <v>81122101</v>
@@ -12172,10 +12172,10 @@
         <v>84</v>
       </c>
       <c r="J228" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="K228" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L228">
         <v>81122101</v>
@@ -12215,10 +12215,10 @@
         <v>84</v>
       </c>
       <c r="J229" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="K229" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L229">
         <v>81122101</v>
@@ -12258,10 +12258,10 @@
         <v>84</v>
       </c>
       <c r="J230" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="K230" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L230">
         <v>81122101</v>
@@ -12301,10 +12301,10 @@
         <v>84</v>
       </c>
       <c r="J231" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="K231" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L231">
         <v>81122101</v>
@@ -12344,10 +12344,10 @@
         <v>84</v>
       </c>
       <c r="J232" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="K232" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L232">
         <v>81122101</v>
@@ -12396,10 +12396,10 @@
         <v>84</v>
       </c>
       <c r="J233" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="K233" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L233">
         <v>81122101</v>
@@ -12439,10 +12439,10 @@
         <v>84</v>
       </c>
       <c r="J234" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="K234" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L234">
         <v>81122101</v>
@@ -12482,10 +12482,10 @@
         <v>84</v>
       </c>
       <c r="J235" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="K235" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L235">
         <v>81122101</v>
@@ -12525,10 +12525,10 @@
         <v>84</v>
       </c>
       <c r="J236" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K236" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L236">
         <v>81122101</v>
@@ -12568,10 +12568,10 @@
         <v>84</v>
       </c>
       <c r="J237" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K237" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L237">
         <v>81122101</v>
@@ -12611,10 +12611,10 @@
         <v>84</v>
       </c>
       <c r="J238" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K238" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L238">
         <v>81122101</v>
@@ -12654,10 +12654,10 @@
         <v>84</v>
       </c>
       <c r="J239" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K239" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L239">
         <v>81122101</v>
@@ -12697,10 +12697,10 @@
         <v>84</v>
       </c>
       <c r="J240" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K240" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L240">
         <v>81122101</v>
@@ -12740,10 +12740,10 @@
         <v>84</v>
       </c>
       <c r="J241" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="K241" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="L241">
         <v>81122101</v>
@@ -12777,10 +12777,10 @@
         <v>454</v>
       </c>
       <c r="J242" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="K242" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L242">
         <v>81124101</v>
@@ -12815,10 +12815,10 @@
         <v>454</v>
       </c>
       <c r="J243" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="K243" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L243">
         <v>81124101</v>
@@ -12853,10 +12853,10 @@
         <v>454</v>
       </c>
       <c r="J244" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="K244" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L244">
         <v>81124101</v>
@@ -12891,10 +12891,10 @@
         <v>454</v>
       </c>
       <c r="J245" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="K245" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L245">
         <v>81124101</v>
@@ -12929,10 +12929,10 @@
         <v>454</v>
       </c>
       <c r="J246" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="K246" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L246">
         <v>81124101</v>
@@ -12967,10 +12967,10 @@
         <v>454</v>
       </c>
       <c r="J247" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="K247" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L247">
         <v>81124101</v>
@@ -13005,10 +13005,10 @@
         <v>454</v>
       </c>
       <c r="J248" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K248" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L248">
         <v>80124101</v>
@@ -13046,10 +13046,10 @@
         <v>454</v>
       </c>
       <c r="J249" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K249" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L249">
         <v>80124101</v>
@@ -13087,10 +13087,10 @@
         <v>454</v>
       </c>
       <c r="J250" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K250" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L250">
         <v>80124101</v>
@@ -13128,10 +13128,10 @@
         <v>454</v>
       </c>
       <c r="J251" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K251" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L251">
         <v>80124101</v>
@@ -13169,10 +13169,10 @@
         <v>454</v>
       </c>
       <c r="J252" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K252" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L252">
         <v>80124101</v>
@@ -13210,10 +13210,10 @@
         <v>454</v>
       </c>
       <c r="J253" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K253" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L253">
         <v>80124101</v>
@@ -13251,10 +13251,10 @@
         <v>454</v>
       </c>
       <c r="J254" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K254" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L254">
         <v>80124101</v>
@@ -13295,10 +13295,10 @@
         <v>454</v>
       </c>
       <c r="J255" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="K255" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L255">
         <v>81124101</v>
@@ -13324,7 +13324,7 @@
         <v>IT-27-15</v>
       </c>
       <c r="E256" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="F256" s="5" t="s">
         <v>48</v>
@@ -13336,10 +13336,10 @@
         <v>454</v>
       </c>
       <c r="J256" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K256" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L256">
         <v>81124101</v>
@@ -13368,7 +13368,7 @@
         <v>IT-27-16</v>
       </c>
       <c r="E257" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="F257" s="5" t="s">
         <v>47</v>
@@ -13380,10 +13380,10 @@
         <v>454</v>
       </c>
       <c r="J257" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K257" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L257">
         <v>81124101</v>
@@ -13412,20 +13412,20 @@
         <v>IT-27-17</v>
       </c>
       <c r="E258" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="F258" s="5" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="H258"/>
       <c r="I258" t="s">
         <v>454</v>
       </c>
       <c r="J258" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K258" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L258">
         <v>81124101</v>
@@ -13463,10 +13463,10 @@
         <v>454</v>
       </c>
       <c r="J259" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K259" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L259">
         <v>80124101</v>
@@ -13507,10 +13507,10 @@
         <v>454</v>
       </c>
       <c r="J260" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K260" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L260">
         <v>81124101</v>
@@ -13551,10 +13551,10 @@
         <v>454</v>
       </c>
       <c r="J261" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K261" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L261">
         <v>80124101</v>
@@ -13595,10 +13595,10 @@
         <v>454</v>
       </c>
       <c r="J262" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K262" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L262">
         <v>80124101</v>
@@ -13639,10 +13639,10 @@
         <v>454</v>
       </c>
       <c r="J263" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K263" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L263">
         <v>80124101</v>
@@ -13683,10 +13683,10 @@
         <v>454</v>
       </c>
       <c r="J264" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K264" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L264">
         <v>81124101</v>
@@ -13724,10 +13724,10 @@
         <v>454</v>
       </c>
       <c r="J265" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K265" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L265">
         <v>80124101</v>
@@ -13765,10 +13765,10 @@
         <v>454</v>
       </c>
       <c r="J266" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K266" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L266">
         <v>90124101</v>
@@ -13806,10 +13806,10 @@
         <v>454</v>
       </c>
       <c r="J267" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K267" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L267">
         <v>81124101</v>
@@ -13847,10 +13847,10 @@
         <v>454</v>
       </c>
       <c r="J268" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K268" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L268">
         <v>80124101</v>
@@ -13888,10 +13888,10 @@
         <v>454</v>
       </c>
       <c r="J269" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K269" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L269">
         <v>90124101</v>
@@ -13929,10 +13929,10 @@
         <v>454</v>
       </c>
       <c r="J270" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K270" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L270">
         <v>81124101</v>
@@ -13973,10 +13973,10 @@
         <v>454</v>
       </c>
       <c r="J271" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K271" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L271">
         <v>80124101</v>
@@ -14017,10 +14017,10 @@
         <v>454</v>
       </c>
       <c r="J272" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K272" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L272">
         <v>80124101</v>
@@ -14061,10 +14061,10 @@
         <v>454</v>
       </c>
       <c r="J273" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K273" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L273">
         <v>80124101</v>
@@ -14105,10 +14105,10 @@
         <v>454</v>
       </c>
       <c r="J274" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K274" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L274">
         <v>80124101</v>
@@ -14149,10 +14149,10 @@
         <v>454</v>
       </c>
       <c r="J275" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K275" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L275">
         <v>80124101</v>
@@ -14193,10 +14193,10 @@
         <v>454</v>
       </c>
       <c r="J276" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K276" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L276">
         <v>80124101</v>
@@ -14235,10 +14235,10 @@
         <v>454</v>
       </c>
       <c r="J277" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K277" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L277">
         <v>80124101</v>
@@ -14279,10 +14279,10 @@
         <v>454</v>
       </c>
       <c r="J278" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K278" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L278">
         <v>81124101</v>
@@ -14323,10 +14323,10 @@
         <v>454</v>
       </c>
       <c r="J279" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K279" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L279">
         <v>81124101</v>
@@ -14358,17 +14358,17 @@
         <v>208</v>
       </c>
       <c r="F280" s="5" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="H280"/>
       <c r="I280" t="s">
         <v>454</v>
       </c>
       <c r="J280" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K280" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L280">
         <v>81124101</v>
@@ -14406,10 +14406,10 @@
         <v>454</v>
       </c>
       <c r="J281" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K281" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L281">
         <v>80124101</v>
@@ -14450,10 +14450,10 @@
         <v>454</v>
       </c>
       <c r="J282" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K282" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L282">
         <v>81124101</v>
@@ -14494,10 +14494,10 @@
         <v>454</v>
       </c>
       <c r="J283" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K283" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L283">
         <v>80124101</v>
@@ -14535,10 +14535,10 @@
         <v>454</v>
       </c>
       <c r="J284" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K284" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L284">
         <v>80124101</v>
@@ -14576,10 +14576,10 @@
         <v>454</v>
       </c>
       <c r="J285" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K285" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L285">
         <v>80124101</v>
@@ -14615,10 +14615,10 @@
         <v>454</v>
       </c>
       <c r="J286" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K286" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L286">
         <v>80124101</v>
@@ -14654,10 +14654,10 @@
         <v>454</v>
       </c>
       <c r="J287" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K287" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L287">
         <v>81124101</v>
@@ -14695,10 +14695,10 @@
         <v>454</v>
       </c>
       <c r="J288" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K288" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L288">
         <v>81124101</v>
@@ -14734,10 +14734,10 @@
         <v>454</v>
       </c>
       <c r="J289" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K289" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L289">
         <v>81124101</v>
@@ -14775,10 +14775,10 @@
         <v>454</v>
       </c>
       <c r="J290" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K290" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L290">
         <v>80124101</v>
@@ -14814,10 +14814,10 @@
         <v>454</v>
       </c>
       <c r="J291" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K291" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L291">
         <v>81124101</v>
@@ -14855,10 +14855,10 @@
         <v>454</v>
       </c>
       <c r="J292" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K292" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L292">
         <v>80124101</v>
@@ -14899,10 +14899,10 @@
         <v>454</v>
       </c>
       <c r="J293" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K293" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L293">
         <v>80124101</v>
@@ -14943,10 +14943,10 @@
         <v>454</v>
       </c>
       <c r="J294" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K294" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L294">
         <v>81124101</v>
@@ -14984,10 +14984,10 @@
         <v>454</v>
       </c>
       <c r="J295" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K295" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L295">
         <v>80124101</v>
@@ -15028,10 +15028,10 @@
         <v>454</v>
       </c>
       <c r="J296" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K296" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L296">
         <v>80124101</v>
@@ -15067,10 +15067,10 @@
         <v>454</v>
       </c>
       <c r="J297" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K297" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L297">
         <v>81124101</v>
@@ -15108,10 +15108,10 @@
         <v>454</v>
       </c>
       <c r="J298" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K298" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L298">
         <v>81124101</v>
@@ -15152,10 +15152,10 @@
         <v>454</v>
       </c>
       <c r="J299" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K299" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L299">
         <v>80124101</v>
@@ -15196,10 +15196,10 @@
         <v>454</v>
       </c>
       <c r="J300" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K300" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L300">
         <v>80124101</v>
@@ -15240,10 +15240,10 @@
         <v>454</v>
       </c>
       <c r="J301" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K301" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L301">
         <v>80124101</v>
@@ -15281,10 +15281,10 @@
         <v>454</v>
       </c>
       <c r="J302" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K302" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L302">
         <v>80124101</v>
@@ -15320,10 +15320,10 @@
         <v>454</v>
       </c>
       <c r="J303" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K303" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L303">
         <v>80124101</v>
@@ -15362,10 +15362,10 @@
         <v>454</v>
       </c>
       <c r="J304" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K304" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L304">
         <v>81124101</v>
@@ -15403,10 +15403,10 @@
         <v>454</v>
       </c>
       <c r="J305" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K305" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L305">
         <v>80124101</v>
@@ -15444,10 +15444,10 @@
         <v>454</v>
       </c>
       <c r="J306" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K306" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L306">
         <v>81124101</v>
@@ -15483,10 +15483,10 @@
         <v>454</v>
       </c>
       <c r="J307" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K307" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L307">
         <v>80124101</v>
@@ -15524,10 +15524,10 @@
         <v>454</v>
       </c>
       <c r="J308" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="K308" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L308">
         <v>81124101</v>
@@ -15559,16 +15559,16 @@
         <v>264</v>
       </c>
       <c r="F309" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="I309" s="5" t="s">
         <v>323</v>
       </c>
       <c r="J309" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K309" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L309">
         <v>90122101</v>
@@ -15605,10 +15605,10 @@
         <v>323</v>
       </c>
       <c r="J310" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K310" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L310">
         <v>80123101</v>
@@ -15649,10 +15649,10 @@
         <v>323</v>
       </c>
       <c r="J311" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K311" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L311">
         <v>90123101</v>
@@ -15693,10 +15693,10 @@
         <v>323</v>
       </c>
       <c r="J312" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K312" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L312">
         <v>81123101</v>
@@ -15734,10 +15734,10 @@
         <v>323</v>
       </c>
       <c r="J313" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K313" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L313">
         <v>80123101</v>
@@ -15775,10 +15775,10 @@
         <v>323</v>
       </c>
       <c r="J314" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K314" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L314">
         <v>80123101</v>
@@ -15816,10 +15816,10 @@
         <v>323</v>
       </c>
       <c r="J315" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K315" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L315">
         <v>80123101</v>
@@ -15857,10 +15857,10 @@
         <v>323</v>
       </c>
       <c r="J316" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K316" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L316">
         <v>80123101</v>
@@ -15898,10 +15898,10 @@
         <v>323</v>
       </c>
       <c r="J317" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K317" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L317">
         <v>80123101</v>
@@ -15933,16 +15933,16 @@
         <v>333</v>
       </c>
       <c r="F318" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="I318" t="s">
         <v>323</v>
       </c>
       <c r="J318" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K318" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L318">
         <v>80123101</v>
@@ -15980,10 +15980,10 @@
         <v>323</v>
       </c>
       <c r="J319" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K319" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L319">
         <v>80123101</v>
@@ -16021,10 +16021,10 @@
         <v>323</v>
       </c>
       <c r="J320" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K320" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L320">
         <v>81123101</v>
@@ -16059,10 +16059,10 @@
         <v>323</v>
       </c>
       <c r="J321" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K321" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L321">
         <v>80123101</v>
@@ -16100,10 +16100,10 @@
         <v>323</v>
       </c>
       <c r="J322" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K322" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L322">
         <v>90123101</v>
@@ -16128,7 +16128,7 @@
         <v>14</v>
       </c>
       <c r="D323" t="str">
-        <f t="shared" ref="D323:D386" si="17">A323&amp;-B323&amp;-C323</f>
+        <f t="shared" ref="D323:D360" si="17">A323&amp;-B323&amp;-C323</f>
         <v>LG-27-14</v>
       </c>
       <c r="E323" t="s">
@@ -16141,10 +16141,10 @@
         <v>323</v>
       </c>
       <c r="J323" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="K323" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L323">
         <v>90122101</v>
@@ -16184,10 +16184,10 @@
         <v>290</v>
       </c>
       <c r="J324" s="5" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K324" s="5" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="L324">
         <v>81111204</v>
@@ -16225,10 +16225,10 @@
         <v>290</v>
       </c>
       <c r="J325" s="5" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K325" s="5" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="L325">
         <v>90111204</v>
@@ -16266,10 +16266,10 @@
         <v>290</v>
       </c>
       <c r="J326" s="5" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K326" s="5" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="L326">
         <v>80111204</v>
@@ -16304,10 +16304,10 @@
         <v>290</v>
       </c>
       <c r="J327" s="5" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K327" s="5" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="L327">
         <v>81134102</v>
@@ -16344,10 +16344,10 @@
         <v>300</v>
       </c>
       <c r="J328" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="K328" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="L328">
         <v>81319101</v>
@@ -16385,10 +16385,10 @@
         <v>300</v>
       </c>
       <c r="J329" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="K329" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="L329">
         <v>81319101</v>
@@ -16426,10 +16426,10 @@
         <v>300</v>
       </c>
       <c r="J330" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="K330" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="L330">
         <v>81319101</v>
@@ -16470,10 +16470,10 @@
         <v>300</v>
       </c>
       <c r="J331" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="K331" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="L331">
         <v>81319101</v>
@@ -16511,10 +16511,10 @@
         <v>300</v>
       </c>
       <c r="J332" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="K332" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="L332">
         <v>81319101</v>
@@ -16552,10 +16552,10 @@
         <v>300</v>
       </c>
       <c r="J333" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="K333" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="L333">
         <v>81319101</v>
@@ -16593,10 +16593,10 @@
         <v>300</v>
       </c>
       <c r="J334" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="K334" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="L334">
         <v>81319101</v>
@@ -16634,10 +16634,10 @@
         <v>300</v>
       </c>
       <c r="J335" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="K335" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="L335">
         <v>81319101</v>
@@ -16669,16 +16669,16 @@
         <v>264</v>
       </c>
       <c r="F336" s="5" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="I336" t="s">
         <v>350</v>
       </c>
       <c r="J336" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="K336" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="L336">
         <v>80133103</v>
@@ -16716,10 +16716,10 @@
         <v>350</v>
       </c>
       <c r="J337" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="K337" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="L337">
         <v>81133103</v>
@@ -16760,10 +16760,10 @@
         <v>350</v>
       </c>
       <c r="J338" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="K338" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="L338">
         <v>80133103</v>
@@ -16804,10 +16804,10 @@
         <v>86</v>
       </c>
       <c r="J339" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K339" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L339">
         <v>80133102</v>
@@ -16849,10 +16849,10 @@
         <v>86</v>
       </c>
       <c r="J340" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K340" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L340">
         <v>81133102</v>
@@ -16891,10 +16891,10 @@
         <v>86</v>
       </c>
       <c r="J341" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K341" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L341">
         <v>90133102</v>
@@ -16931,10 +16931,10 @@
         <v>86</v>
       </c>
       <c r="J342" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K342" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L342">
         <v>80133102</v>
@@ -16976,10 +16976,10 @@
         <v>86</v>
       </c>
       <c r="J343" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K343" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L343">
         <v>80111101</v>
@@ -17021,10 +17021,10 @@
         <v>86</v>
       </c>
       <c r="J344" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K344" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L344">
         <v>81111101</v>
@@ -17066,10 +17066,10 @@
         <v>86</v>
       </c>
       <c r="J345" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K345" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L345">
         <v>90111101</v>
@@ -17111,10 +17111,10 @@
         <v>86</v>
       </c>
       <c r="J346" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K346" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L346">
         <v>90111101</v>
@@ -17156,10 +17156,10 @@
         <v>86</v>
       </c>
       <c r="J347" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K347" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L347">
         <v>80111101</v>
@@ -17201,10 +17201,10 @@
         <v>86</v>
       </c>
       <c r="J348" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K348" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L348">
         <v>81111101</v>
@@ -17246,10 +17246,10 @@
         <v>86</v>
       </c>
       <c r="J349" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K349" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L349">
         <v>90111101</v>
@@ -17291,10 +17291,10 @@
         <v>86</v>
       </c>
       <c r="J350" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K350" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L350">
         <v>90111101</v>
@@ -17336,10 +17336,10 @@
         <v>86</v>
       </c>
       <c r="J351" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K351" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L351">
         <v>81111101</v>
@@ -17381,10 +17381,10 @@
         <v>86</v>
       </c>
       <c r="J352" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K352" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L352">
         <v>90111101</v>
@@ -17426,10 +17426,10 @@
         <v>86</v>
       </c>
       <c r="J353" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K353" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L353">
         <v>90111101</v>
@@ -17471,10 +17471,10 @@
         <v>86</v>
       </c>
       <c r="J354" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K354" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L354">
         <v>80133102</v>
@@ -17516,10 +17516,10 @@
         <v>86</v>
       </c>
       <c r="J355" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K355" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L355">
         <v>81133102</v>
@@ -17561,10 +17561,10 @@
         <v>86</v>
       </c>
       <c r="J356" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K356" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L356">
         <v>90133102</v>
@@ -17596,16 +17596,16 @@
         <v>247</v>
       </c>
       <c r="F357" s="5" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="I357" t="s">
         <v>86</v>
       </c>
       <c r="J357" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K357" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L357">
         <v>90133102</v>
@@ -17634,7 +17634,7 @@
         <v>247</v>
       </c>
       <c r="F358" s="5" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="G358" s="5" t="s">
         <v>220</v>
@@ -17643,10 +17643,10 @@
         <v>86</v>
       </c>
       <c r="J358" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K358" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L358">
         <v>80111101</v>
@@ -17675,7 +17675,7 @@
         <v>247</v>
       </c>
       <c r="F359" s="5" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="G359" s="5" t="s">
         <v>221</v>
@@ -17684,10 +17684,10 @@
         <v>86</v>
       </c>
       <c r="J359" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K359" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L359">
         <v>81111101</v>
@@ -17716,16 +17716,16 @@
         <v>325</v>
       </c>
       <c r="F360" s="5" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="I360" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="J360" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="K360" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="L360">
         <v>80215106</v>
@@ -17736,7 +17736,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A2:R360" xr:uid="{0B1226CB-0107-4D8F-A599-9B58ED89F844}"/>
-  <conditionalFormatting sqref="J225:J235 H2:H202 H209:H1048576 J152:J213 J118:J140 K50:K80 J36:K49">
+  <conditionalFormatting sqref="J225:J235 H2:H202 H209:H1048576 J158:J213 K50:K80 J36:K49">
     <cfRule type="duplicateValues" dxfId="0" priority="23"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17851,10 +17851,10 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B14" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
   </sheetData>

</xml_diff>